<commit_message>
Changes done as per required
</commit_message>
<xml_diff>
--- a/src/main/resources/FundingSource_Field_Values.xlsx
+++ b/src/main/resources/FundingSource_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF45E929-E8E7-4C82-8237-5FD9BAB938F4}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F61F8975-DE9D-4093-B856-B92D75160746}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="23">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -459,14 +459,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F0A2B2E-B537-4457-8666-B87F52CC4438}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -477,7 +477,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -486,6 +486,28 @@
       </c>
       <c r="C2" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4">
+        <v>760</v>
       </c>
     </row>
   </sheetData>
@@ -495,14 +517,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{542C2F33-0CA3-46B6-B0DA-5252E99270E2}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -513,26 +535,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3">
-        <v>760</v>
+        <v>761</v>
       </c>
     </row>
   </sheetData>
@@ -542,14 +553,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA8F565D-4A1E-40DC-8370-113D6BE62705}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="51.33203125" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -560,7 +571,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -571,7 +582,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -580,6 +591,17 @@
       </c>
       <c r="C3" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4">
+        <v>10000000</v>
       </c>
     </row>
   </sheetData>
@@ -589,14 +611,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F784967-C83D-450C-97CE-71BB91D2ED97}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5546875" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -607,7 +629,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -618,7 +640,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -629,7 +651,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -640,7 +662,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -651,7 +673,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -662,7 +684,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -673,7 +695,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -682,17 +704,6 @@
       </c>
       <c r="C8" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9">
-        <v>10000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Merged PR 2631: Merge MahadevProductB to master
refactored planning and payment request module
</commit_message>
<xml_diff>
--- a/src/main/resources/FundingSource_Field_Values.xlsx
+++ b/src/main/resources/FundingSource_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{201C5F30-F99D-4727-B373-BDC093C4451D}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7632C419-69F9-4CE7-9C65-50AFB3C33999}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -461,13 +461,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F0A2B2E-B537-4457-8666-B87F52CC4438}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -478,7 +478,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -489,7 +489,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -497,10 +497,10 @@
         <v>5</v>
       </c>
       <c r="C3">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -520,13 +520,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{542C2F33-0CA3-46B6-B0DA-5252E99270E2}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -537,7 +537,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -556,13 +556,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA8F565D-4A1E-40DC-8370-113D6BE62705}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="24.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="51.33203125" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -573,7 +573,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -584,7 +584,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -595,7 +595,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -615,13 +615,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F784967-C83D-450C-97CE-71BB91D2ED97}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5546875" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -632,7 +632,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -640,10 +640,10 @@
         <v>5</v>
       </c>
       <c r="C2">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -651,10 +651,10 @@
         <v>7</v>
       </c>
       <c r="C3">
-        <v>761</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -665,7 +665,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -676,7 +676,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -687,7 +687,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -698,7 +698,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 2734: Merge MahadevProductB to master
Done fixes in test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/FundingSource_Field_Values.xlsx
+++ b/src/main/resources/FundingSource_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7632C419-69F9-4CE7-9C65-50AFB3C33999}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B528B5-C65B-4FA7-B4DE-4B3B78655F60}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -497,7 +497,7 @@
         <v>5</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -508,7 +508,7 @@
         <v>7</v>
       </c>
       <c r="C4">
-        <v>761</v>
+        <v>3650</v>
       </c>
     </row>
   </sheetData>
@@ -640,7 +640,7 @@
         <v>5</v>
       </c>
       <c r="C2">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -651,7 +651,7 @@
         <v>7</v>
       </c>
       <c r="C3">
-        <v>750</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Merged PR 3005: Merge mhomefixes to master-grey
Updated test cases as per QA org
</commit_message>
<xml_diff>
--- a/src/main/resources/FundingSource_Field_Values.xlsx
+++ b/src/main/resources/FundingSource_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21901"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B528B5-C65B-4FA7-B4DE-4B3B78655F60}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC0EEAE-5438-4A50-BB9B-F1ADA47E7372}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -545,7 +545,7 @@
         <v>7</v>
       </c>
       <c r="C2">
-        <v>761</v>
+        <v>3650</v>
       </c>
     </row>
   </sheetData>
@@ -640,7 +640,7 @@
         <v>5</v>
       </c>
       <c r="C2">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fixed business flow for kpi, announcement and application
</commit_message>
<xml_diff>
--- a/src/main/resources/FundingSource_Field_Values.xlsx
+++ b/src/main/resources/FundingSource_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\REI_Automation_Project\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC0EEAE-5438-4A50-BB9B-F1ADA47E7372}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B395C4-9344-40CA-A023-B51D3A9A22BD}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" activeTab="3" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -461,13 +461,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F0A2B2E-B537-4457-8666-B87F52CC4438}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.3046875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -478,7 +478,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -489,7 +489,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -500,7 +500,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -520,13 +520,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{542C2F33-0CA3-46B6-B0DA-5252E99270E2}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -537,7 +537,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -556,13 +556,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA8F565D-4A1E-40DC-8370-113D6BE62705}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="51.28515625" customWidth="1"/>
+    <col min="2" max="2" width="24.3828125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51.3046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -573,7 +573,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -584,7 +584,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -595,7 +595,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -615,13 +615,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F784967-C83D-450C-97CE-71BB91D2ED97}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5703125" customWidth="1"/>
+    <col min="2" max="2" width="21.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -632,7 +632,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -640,10 +640,10 @@
         <v>5</v>
       </c>
       <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -654,7 +654,7 @@
         <v>2650</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -665,7 +665,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -676,7 +676,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -687,7 +687,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -698,7 +698,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 3016: Merge pr2_testcases to master-grey
1. Added code to initialize the data such as funding account which can be different based on environment(Can be use to any kind of data)
2. This will make refactoring easier.
</commit_message>
<xml_diff>
--- a/src/main/resources/FundingSource_Field_Values.xlsx
+++ b/src/main/resources/FundingSource_Field_Values.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\REI_Automation_Project\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC0EEAE-5438-4A50-BB9B-F1ADA47E7372}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B395C4-9344-40CA-A023-B51D3A9A22BD}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" activeTab="3" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -461,13 +461,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F0A2B2E-B537-4457-8666-B87F52CC4438}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.3046875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -478,7 +478,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -489,7 +489,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -500,7 +500,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -520,13 +520,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{542C2F33-0CA3-46B6-B0DA-5252E99270E2}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -537,7 +537,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -556,13 +556,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA8F565D-4A1E-40DC-8370-113D6BE62705}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="51.28515625" customWidth="1"/>
+    <col min="2" max="2" width="24.3828125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51.3046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -573,7 +573,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -584,7 +584,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -595,7 +595,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -615,13 +615,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F784967-C83D-450C-97CE-71BB91D2ED97}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5703125" customWidth="1"/>
+    <col min="2" max="2" width="21.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -632,7 +632,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -640,10 +640,10 @@
         <v>5</v>
       </c>
       <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -654,7 +654,7 @@
         <v>2650</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -665,7 +665,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -676,7 +676,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -687,7 +687,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -698,7 +698,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
Merged PR 3035: Merge DeepikaNewTestCasesMain to master
Fixed Test Cases
</commit_message>
<xml_diff>
--- a/src/main/resources/FundingSource_Field_Values.xlsx
+++ b/src/main/resources/FundingSource_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21901"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace-Product-Automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B528B5-C65B-4FA7-B4DE-4B3B78655F60}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEC0EEAE-5438-4A50-BB9B-F1ADA47E7372}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -545,7 +545,7 @@
         <v>7</v>
       </c>
       <c r="C2">
-        <v>761</v>
+        <v>3650</v>
       </c>
     </row>
   </sheetData>
@@ -640,7 +640,7 @@
         <v>5</v>
       </c>
       <c r="C2">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
updated program test cases : with new api approach
</commit_message>
<xml_diff>
--- a/src/main/resources/FundingSource_Field_Values.xlsx
+++ b/src/main/resources/FundingSource_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22624"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\Automation projects\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF7F48DD-1451-4319-B17A-37F9BE5F471B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{112C2525-684A-4338-9BC5-7F5708B8373E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" activeTab="2" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -86,16 +86,16 @@
     <t>AppropriationBalance__c</t>
   </si>
   <si>
-    <t>Automation Execution Funding Account</t>
-  </si>
-  <si>
     <t>Funding Source Description</t>
   </si>
   <si>
     <t>Description__c</t>
   </si>
   <si>
-    <t>Automation Execution Funding Source</t>
+    <t>Automation Runtime Funding Source</t>
+  </si>
+  <si>
+    <t>Automation Runtime Funding Account</t>
   </si>
 </sst>
 </file>
@@ -455,13 +455,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F0A2B2E-B537-4457-8666-B87F52CC4438}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.3046875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -472,7 +472,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -480,10 +480,10 @@
         <v>4</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -494,7 +494,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -514,13 +514,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{542C2F33-0CA3-46B6-B0DA-5252E99270E2}">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -531,7 +531,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -550,13 +550,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA8F565D-4A1E-40DC-8370-113D6BE62705}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="51.33203125" customWidth="1"/>
+    <col min="2" max="2" width="24.3046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51.3046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -567,7 +567,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -575,21 +575,21 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -609,13 +609,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F784967-C83D-450C-97CE-71BB91D2ED97}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5546875" customWidth="1"/>
+    <col min="2" max="2" width="21.84375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -626,7 +626,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -637,7 +637,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -648,7 +648,7 @@
         <v>2650</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -659,7 +659,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -670,7 +670,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -681,7 +681,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
Again modification as per execution report (Second day)
</commit_message>
<xml_diff>
--- a/src/main/resources/FundingSource_Field_Values.xlsx
+++ b/src/main/resources/FundingSource_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22624"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\Automation projects\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{112C2525-684A-4338-9BC5-7F5708B8373E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A31296A4-8AB2-4817-944C-1C566CC81369}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" activeTab="2" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{11C5240F-7765-4FC9-A357-1384C2AAB3E6}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="23">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -96,19 +96,31 @@
   </si>
   <si>
     <t>Automation Runtime Funding Account</t>
+  </si>
+  <si>
+    <t>fieldEndDate__c</t>
+  </si>
+  <si>
+    <t>fieldStartDate__c</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="5"/>
+      <color rgb="FF222222"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -131,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -140,6 +152,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -455,13 +468,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F0A2B2E-B537-4457-8666-B87F52CC4438}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="13.3046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -472,7 +485,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -483,7 +496,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -494,7 +507,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -513,14 +526,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{542C2F33-0CA3-46B6-B0DA-5252E99270E2}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="13.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.69140625" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -531,32 +544,44 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
-        <v>7</v>
+      <c r="B2" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="C2">
         <v>3650</v>
       </c>
     </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA8F565D-4A1E-40DC-8370-113D6BE62705}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="24.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="51.3046875" customWidth="1"/>
+    <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="51.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -567,7 +592,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -578,7 +603,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -589,7 +614,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -609,13 +634,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F784967-C83D-450C-97CE-71BB91D2ED97}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="21.84375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.53515625" customWidth="1"/>
+    <col min="2" max="2" width="21.86328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -626,7 +651,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -637,7 +662,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -648,7 +673,7 @@
         <v>2650</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -659,7 +684,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -670,7 +695,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -681,7 +706,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>6</v>
       </c>

</xml_diff>